<commit_message>
zeros for offshore storage nodes
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/import_export/ImportExport_unlimited_2040.xlsx
+++ b/mes_north_sea/clean_data/import_export/ImportExport_unlimited_2040.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\6574114\PycharmProjects\PyHubProductive\mes_north_sea\clean_data\import_export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData-maian_NS_final/mes_north_sea/clean_data/import_export/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB0E70D-C717-4A09-AEBE-DFCDEDDCC08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89360C16-A585-FD44-9AD8-6659683AB946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-240" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>Import_electricity</t>
   </si>
@@ -222,6 +222,15 @@
   </si>
   <si>
     <t>DE_G</t>
+  </si>
+  <si>
+    <t>NO_ST1</t>
+  </si>
+  <si>
+    <t>NO_ST2</t>
+  </si>
+  <si>
+    <t>DK_ST1</t>
   </si>
 </sst>
 </file>
@@ -539,10 +548,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -565,7 +574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -588,7 +597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -611,7 +620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -634,7 +643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -657,7 +666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -680,7 +689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -703,7 +712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -726,7 +735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -749,7 +758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -772,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -795,7 +804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -818,7 +827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -841,7 +850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -864,7 +873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -887,7 +896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -910,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -933,7 +942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -956,7 +965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -979,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1002,7 +1011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1025,7 +1034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -1048,7 +1057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1071,7 +1080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1094,7 +1103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -1117,7 +1126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1140,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1163,7 +1172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -1186,7 +1195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1209,7 +1218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1232,7 +1241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1255,7 +1264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1278,7 +1287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -1301,7 +1310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -1324,7 +1333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -1347,7 +1356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -1370,7 +1379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -1393,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -1416,7 +1425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -1439,7 +1448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -1462,7 +1471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -1485,7 +1494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -1508,7 +1517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -1531,7 +1540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1554,7 +1563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -1577,7 +1586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -1600,7 +1609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1623,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -1646,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -1669,7 +1678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -1692,7 +1701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -1715,7 +1724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -1738,7 +1747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -1761,7 +1770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -1784,7 +1793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -1807,7 +1816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -1827,6 +1836,75 @@
         <v>0</v>
       </c>
       <c r="G56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57">
+        <v>0</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>63</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
         <v>0</v>
       </c>
     </row>

</xml_diff>